<commit_message>
Update 96-well map and add example spreadsheets
</commit_message>
<xml_diff>
--- a/examples/data/96WellPlateMap_PBSouter_20260216_021203.xlsx
+++ b/examples/data/96WellPlateMap_PBSouter_20260216_021203.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Caleb\Documents\GitHub\jaegertros\illucidate\examples\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{595F9A9E-38F6-4444-87BE-1F874E8109EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{435BA7E2-26FC-452F-97BD-53BCE48AB351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B8146891-5002-489B-B1AE-C68553CF2933}"/>
   </bookViews>
@@ -79,14 +79,6 @@
     <t>250 µL PBS</t>
   </si>
   <si>
-    <t>240  µL LB:
-10 uL substrate</t>
-  </si>
-  <si>
-    <t>240  µL C7927:
-10 uL substrate</t>
-  </si>
-  <si>
     <t>240  µL -3 C7927;
 10 uL H2O</t>
   </si>
@@ -126,6 +118,14 @@
   <si>
     <t>60  µL -4 NanoLuc;
 180  µL -4 O157 lux;
+10 uL substrate</t>
+  </si>
+  <si>
+    <t>240  µL C7927;
+10 uL substrate</t>
+  </si>
+  <si>
+    <t>240  µL LB;
 10 uL substrate</t>
   </si>
 </sst>
@@ -702,34 +702,34 @@
         <v>9</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="M3" t="s">
         <v>9</v>
@@ -746,34 +746,34 @@
         <v>9</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="M4" t="s">
         <v>9</v>
@@ -790,34 +790,34 @@
         <v>9</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L5" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="M5" t="s">
         <v>9</v>
@@ -834,34 +834,34 @@
         <v>8</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M6" t="s">
         <v>9</v>
@@ -878,34 +878,34 @@
         <v>9</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L7" s="9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="M7" t="s">
         <v>9</v>
@@ -922,34 +922,34 @@
         <v>9</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="M8" t="s">
         <v>9</v>

</xml_diff>